<commit_message>
fix(news): update 2026-10-23 verified coverage typography
</commit_message>
<xml_diff>
--- a/docs/exports/day-2026-10-23.xlsx
+++ b/docs/exports/day-2026-10-23.xlsx
@@ -119,7 +119,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="98" customHeight="1">
+    <row r="3" ht="134" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">01</t>
@@ -134,16 +134,16 @@
               <rFont val="PingFang TC"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">NVIDIA公布京元電11億美元預付款，矽品光學引擎規劃增產15倍
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="PingFang TC"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">NVIDIA 10月21日在柏林GTC宣布，規劃以11億美元測試產能預訂預付款支持京元電美國新廠，目標2027年4月量產；矽品台灣CPO光學引擎產能目標2027年中提升至現有15倍。欣興台灣KF載板擴產預定2027年第2季起增加產能，均為未來計畫。</t>
+            <t xml:space="preserve">NVIDIA 公布京元電 11 億美元預付款，矽品光學引擎規劃增產 15 倍
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="PingFang TC"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">NVIDIA 10 月 21 日在柏林 GTC 宣布，規劃以 11 億美元測試產能預訂預付款支持京元電美國新廠，目標 2027 年 4 月量產；矽品台灣 CPO 光學引擎產能目標 2027 年中提升至現有 15 倍。欣興台灣 KF 載板擴產預定 2027 年第 2 季起增加產能，均為未來計畫。</t>
           </r>
         </is>
       </c>
@@ -151,7 +151,7 @@
         <v>46316</v>
       </c>
     </row>
-    <row r="4" ht="82" customHeight="1">
+    <row r="4" ht="98" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">02</t>
@@ -166,16 +166,16 @@
               <rFont val="PingFang TC"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">聯電與愛普合作矽電容，Gen2D已完成投片和初步驗證
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="PingFang TC"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">聯電與愛普10月22日在新竹宣布深溝槽電容（DTC）晶圓製造與S-SiCap矽電容設計合作。愛普Gen2D產品已於第三季完成投片和初步功能驗證，後續將進行封裝基板系統級效能與可靠度測試；雙方尚未宣布客戶量產驗收。</t>
+            <t xml:space="preserve">聯電與愛普合作矽電容，Gen2D 已完成投片和初步驗證
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="PingFang TC"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">聯電與愛普 10 月 22 日在新竹宣布深溝槽電容（DTC）晶圓製造與 S-SiCap 矽電容設計合作。愛普 Gen2D 產品已於第三季完成投片和初步功能驗證，後續將進行封裝基板系統級效能與可靠度測試；雙方尚未宣布客戶量產驗收。</t>
           </r>
         </is>
       </c>
@@ -183,7 +183,7 @@
         <v>46317</v>
       </c>
     </row>
-    <row r="5" ht="82" customHeight="1">
+    <row r="5" ht="98" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">03</t>
@@ -198,16 +198,16 @@
               <rFont val="PingFang TC"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">追蹤：美光桃園11名工會幹部罷工，公布季度分潤及勞退調升
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="PingFang TC"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">美光桃園工會11名幹部10月22日上午9時起展開24小時罷工，台中工會則已於前一天達成協議。美光同日公布季度分潤獎金採現金與股票各半，台灣員工勞退提撥率由8%提高至10%，並增3天有薪假；實際產線損失仍未披露。</t>
+            <t xml:space="preserve">追蹤：美光桃園 11 名工會幹部罷工，公布季度分潤及勞退調升
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="PingFang TC"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">美光桃園工會 11 名幹部 10 月 22 日上午 9 時起展開 24 小時罷工，台中工會則已於前一天達成協議。美光同日公布季度分潤獎金採現金與股票各半，台灣員工勞退提撥率由 8% 提高至 10%，並增 3 天有薪假；實際產線損失仍未披露。</t>
           </r>
         </is>
       </c>
@@ -239,7 +239,7 @@
               <rFont val="PingFang TC"/>
               <color rgb="FF3B4A44"/>
             </rPr>
-            <t xml:space="preserve">Reuters 10月22日引述3名知情人士指出，台積電正調查半導體自動化設備使用低稀土或無稀土馬達的可能性，以降低部分設備供應受出口管制影響。報導指出供應商洽詢尚處早期，未有廣泛導入；台積電拒絕評論。</t>
+            <t xml:space="preserve">Reuters 10 月 22 日引述 3 名知情人士指出，台積電正調查半導體自動化設備使用低稀土或無稀土馬達的可能性，以降低部分設備供應受出口管制影響。報導指出供應商洽詢尚處早期，未有廣泛導入；台積電拒絕評論。</t>
           </r>
         </is>
       </c>
@@ -247,7 +247,7 @@
         <v>46317</v>
       </c>
     </row>
-    <row r="7" ht="118" customHeight="1">
+    <row r="7" ht="134" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">05</t>
@@ -262,16 +262,16 @@
               <rFont val="PingFang TC"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">NVIDIA推出DSX POD模組化AI機房，鴻海與台灣ODM列合作供應商
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="PingFang TC"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">NVIDIA 10月21日在德國柏林公布以Vera Rubin為核心的DSX POD模組化AI工廠參考設計，合作廠商包括鴻海鴻佰、台達電、技嘉、和碩、雲達及緯創。NVIDIA稱已備妥現場基礎設施的案場部署可由6個月縮短至最快14天，全球合作交付目標為2027年初。</t>
+            <t xml:space="preserve">NVIDIA 推出 DSX POD 模組化 AI 機房，鴻海與台灣 ODM 列合作供應商
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="PingFang TC"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">NVIDIA 10 月 21 日在德國柏林公布以 Vera Rubin 為核心的 DSX POD 模組化 AI 工廠參考設計，合作廠商包括鴻海鴻佰、台達電、技嘉、和碩、雲達及緯創。NVIDIA 稱已備妥現場基礎設施的案場部署可由 6 個月縮短至最快 14 天，全球合作交付目標為 2027 年初。</t>
           </r>
         </is>
       </c>
@@ -294,16 +294,16 @@
               <rFont val="PingFang TC"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">馬來西亞SkyeChip與日本SAIMEMORY合作ZAM新型AI記憶體設計
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="PingFang TC"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">日本SAIMEMORY與馬來西亞SkyeChip於10月21日宣布設計工程合作，由SkyeChip提供記憶體介面、矽晶片設計及客製化IP，參與面向AI資料中心的Z-Angle Memory（ZAM）開發。官方公告未提供原型測試結果、記憶體頻寬或量產時程。</t>
+            <t xml:space="preserve">馬來西亞 SkyeChip 與日本 SAIMEMORY 合作 ZAM 新型 AI 記憶體設計
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="PingFang TC"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">日本 SAIMEMORY 與馬來西亞 SkyeChip 於 10 月 21 日宣布設計工程合作，由 SkyeChip 提供記憶體介面、矽晶片設計及客製化 IP，參與面向 AI 資料中心的 Z-Angle Memory（ZAM）開發。官方公告未提供原型測試結果、記憶體頻寬或量產時程。</t>
           </r>
         </is>
       </c>
@@ -326,16 +326,16 @@
               <rFont val="PingFang TC"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">台綜院：9月半導體用電首破45億度，年增11.55%
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="PingFang TC"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">台灣綜合研究院10月21日公布，2026年9月台灣半導體業用電量首次突破45億度，較去年同期增加11.55%；製造業高壓以上用電年增1.96%。台綜院預估全年半導體用電超過500億度，屬研究機構估計，並非全年已發生實績。</t>
+            <t xml:space="preserve">台綜院：9 月半導體用電首破 45 億度，年增 11.55%
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="PingFang TC"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">台灣綜合研究院 10 月 21 日公布，2026 年 9 月台灣半導體業用電量首次突破 45 億度，較去年同期增加 11.55%；製造業高壓以上用電年增 1.96%。台綜院預估全年半導體用電超過 500 億度，屬研究機構估計，並非全年已發生實績。</t>
           </r>
         </is>
       </c>
@@ -343,7 +343,7 @@
         <v>46316</v>
       </c>
     </row>
-    <row r="10" ht="98" customHeight="1">
+    <row r="10" ht="114" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">08</t>
@@ -358,16 +358,16 @@
               <rFont val="PingFang TC"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">馬國國會披露半導體培訓核准4,767萬令吉，涵蓋1.9萬名額
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="PingFang TC"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">馬來西亞貿工部長10月22日經媒體報導向國會指出，HRD Corp已於8月核准4,767萬令吉高科技培訓補助，涵蓋19,084個名額及9類半導體相關技能。截至2026年第3季，累計已有22,849名勞工完成各項相關訓練；這些數字各屬不同統計期間，不能直接相減作為未完成名額。</t>
+            <t xml:space="preserve">馬國國會披露半導體培訓核准 4,767 萬令吉，涵蓋 1.9 萬名額
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="PingFang TC"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">馬來西亞貿工部長 10 月 22 日經媒體報導向國會指出，HRD Corp 已於 8 月核准 4,767 萬令吉高科技培訓補助，涵蓋 19,084 個名額及 9 類半導體相關技能。截至 2026 年第 3 季，累計已有 22,849 名勞工完成各項相關訓練；這些數字各屬不同統計期間，不能直接相減作為未完成名額。</t>
           </r>
         </is>
       </c>
@@ -421,7 +421,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="210" customHeight="1">
+    <row r="3" ht="246" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">01</t>
@@ -436,16 +436,16 @@
               <rFont val="PingFang TC"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">NVIDIA公布京元電11億美元預付款，矽品光學引擎規劃增產15倍
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="PingFang TC"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">NVIDIA 10月21日在柏林GTC宣布，規劃以11億美元測試產能預訂預付款支持京元電美國新廠，目標2027年4月量產；矽品台灣CPO光學引擎產能目標2027年中提升至現有15倍。欣興台灣KF載板擴產預定2027年第2季起增加產能，均為未來計畫。公告跨越晶片載板、晶圓級封裝、測試與光學引擎。京元電提供晶片測試，矽品負責CPO光學引擎，欣興提供先進封裝載板；NVIDIA並預期2027年集團半導體測試產能較2026年翻倍，包含美國、台灣與新加坡擴充。NVIDIA表示新加坡測試產能計畫2027年2月開始大規模生產；矽品產能於2028年底前另力求再翻倍。與京元電的11億美元為產能預訂預付款，不能列為已完成廠房投資或公司營收。各項基準月產量、設備到廠、客戶驗收、實際預付款撥付與投產率未公布。地點：德國柏林 GTC 會議（發布活動）；台灣、美國與新加坡擴建廠址尚無完整地點明細。</t>
+            <t xml:space="preserve">NVIDIA 公布京元電 11 億美元預付款，矽品光學引擎規劃增產 15 倍
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="PingFang TC"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">NVIDIA 10 月 21 日在柏林 GTC 宣布，規劃以 11 億美元測試產能預訂預付款支持京元電美國新廠，目標 2027 年 4 月量產；矽品台灣 CPO 光學引擎產能目標 2027 年中提升至現有 15 倍。欣興台灣 KF 載板擴產預定 2027 年第 2 季起增加產能，均為未來計畫。公告跨越晶片載板、晶圓級封裝、測試與光學引擎。京元電提供晶片測試，矽品負責 CPO 光學引擎，欣興提供先進封裝載板；NVIDIA 並預期 2027 年集團半導體測試產能較 2026 年翻倍，包含美國、台灣與新加坡擴充。NVIDIA 表示新加坡測試產能計畫 2027 年 2 月開始大規模生產；矽品產能於 2028 年底前另力求再翻倍。與京元電的 11 億美元為產能預訂預付款，不能列為已完成廠房投資或公司營收。各項基準月產量、設備到廠、客戶驗收、實際預付款撥付與投產率未公布。地點：德國柏林 GTC 會議（發布活動）；台灣、美國與新加坡擴建廠址尚無完整地點明細。</t>
           </r>
         </is>
       </c>
@@ -454,7 +454,7 @@
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">對封測機台、測試量測、基板製程電源與光學模組供應商而言，可核對2027年京元電設備裝機、矽品CPO光學引擎合格產出及欣興KF載板認證節點。公告未提供基準產出和最終採購量，無法從倍率推算設備需求。</t>
+          <t xml:space="preserve">對封測機台、測試量測、基板製程電源與光學模組供應商而言，可核對 2027 年京元電設備裝機、矽品 CPO 光學引擎合格產出及欣興 KF 載板認證節點。公告未提供基準產出和最終採購量，無法從倍率推算設備需求。</t>
         </is>
       </c>
     </row>
@@ -473,16 +473,16 @@
               <rFont val="PingFang TC"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">聯電與愛普合作矽電容，Gen2D已完成投片和初步驗證
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="PingFang TC"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">聯電與愛普10月22日在新竹宣布深溝槽電容（DTC）晶圓製造與S-SiCap矽電容設計合作。愛普Gen2D產品已於第三季完成投片和初步功能驗證，後續將進行封裝基板系統級效能與可靠度測試；雙方尚未宣布客戶量產驗收。DTC矽電容可配置於晶片附近、中介層、封裝基板或封裝底部，降低供電路徑阻抗，與既有PCB上的穩壓元件形成不同整合層級。這項合作連結晶圓代工、先進封裝、電容元件與資料中心晶片供電完整性。聯電提供可擴充晶圓製程，愛普提供客製化矽電容與系統整合。公司表示也在探索內埋中介層電容及封裝底部電容產品線；相關新製造投資尚未公布金額。系統級測試結果、耐壓電容規格、量產良率、客戶導入時點與擴建金額未公布。</t>
+            <t xml:space="preserve">聯電與愛普合作矽電容，Gen2D 已完成投片和初步驗證
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="PingFang TC"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">聯電與愛普 10 月 22 日在新竹宣布深溝槽電容（DTC）晶圓製造與 S-SiCap 矽電容設計合作。愛普 Gen2D 產品已於第三季完成投片和初步功能驗證，後續將進行封裝基板系統級效能與可靠度測試；雙方尚未宣布客戶量產驗收。DTC 矽電容可配置於晶片附近、中介層、封裝基板或封裝底部，降低供電路徑阻抗，與既有 PCB 上的穩壓元件形成不同整合層級。這項合作連結晶圓代工、先進封裝、電容元件與資料中心晶片供電完整性。聯電提供可擴充晶圓製程，愛普提供客製化矽電容與系統整合。公司表示也在探索內埋中介層電容及封裝底部電容產品線；相關新製造投資尚未公布金額。系統級測試結果、耐壓電容規格、量產良率、客戶導入時點與擴建金額未公布。</t>
           </r>
         </is>
       </c>
@@ -491,11 +491,11 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">對電源轉換、晶圓製程與封裝量測業者，值得核對DTC的電壓規格、可靠度測試方法、封裝整合良率和客戶設計導入狀況。目前沒有量產承諾或交貨量可判斷後續需求。</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="178" customHeight="1">
+          <t xml:space="preserve">對電源轉換、晶圓製程與封裝量測業者，值得核對 DTC 的電壓規格、可靠度測試方法、封裝整合良率和客戶設計導入狀況。目前沒有量產承諾或交貨量可判斷後續需求。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="194" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">03</t>
@@ -510,16 +510,16 @@
               <rFont val="PingFang TC"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">追蹤：美光桃園11名工會幹部罷工，公布季度分潤及勞退調升
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="PingFang TC"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">美光桃園工會11名幹部10月22日上午9時起展開24小時罷工，台中工會則已於前一天達成協議。美光同日公布季度分潤獎金採現金與股票各半，台灣員工勞退提撥率由8%提高至10%，並增3天有薪假；實際產線損失仍未披露。桃園廠牽涉DRAM前段晶圓製造，台中廠有先進DRAM、HBM與封裝測試。工會幹部參與行動的實際規模，不能直接推算成整座晶圓廠停產時間。美光管理階層表示本次協議新增季度分潤，現金部分於每季財報後發放，股票獎勵一年後歸屬。公司亦公布輪班津貼和結構性調薪調整，桃園工會仍要求持續對話。未公布工廠產能利用率、實際出貨損失、桃園工會是否接受新方案及台中協議條款全文。地點：台灣桃園美光工廠外（實際工會行動地點，依中央社報導）。</t>
+            <t xml:space="preserve">追蹤：美光桃園 11 名工會幹部罷工，公布季度分潤及勞退調升
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="PingFang TC"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">美光桃園工會 11 名幹部 10 月 22 日上午 9 時起展開 24 小時罷工，台中工會則已於前一天達成協議。美光同日公布季度分潤獎金採現金與股票各半，台灣員工勞退提撥率由 8% 提高至 10%，並增 3 天有薪假；實際產線損失仍未披露。桃園廠牽涉 DRAM 前段晶圓製造，台中廠有先進 DRAM、HBM 與封裝測試。工會幹部參與行動的實際規模，不能直接推算成整座晶圓廠停產時間。美光管理階層表示本次協議新增季度分潤，現金部分於每季財報後發放，股票獎勵一年後歸屬。公司亦公布輪班津貼和結構性調薪調整，桃園工會仍要求持續對話。未公布工廠產能利用率、實際出貨損失、桃園工會是否接受新方案及台中協議條款全文。地點：台灣桃園美光工廠外（實際工會行動地點，依中央社報導）。</t>
           </r>
         </is>
       </c>
@@ -528,7 +528,7 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">製程電源與記憶體測試供應商可核實罷工當日的輪班覆蓋、設備維護及在製品狀態，並留意薪酬協商對工廠排程是否有具體變動。現階段11名工會幹部的行動不足以估算設備需求或良率影響。</t>
+          <t xml:space="preserve">製程電源與記憶體測試供應商可核實罷工當日的輪班覆蓋、設備維護及在製品狀態，並留意薪酬協商對工廠排程是否有具體變動。現階段 11 名工會幹部的行動不足以估算設備需求或良率影響。</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
               <rFont val="PingFang TC"/>
               <color rgb="FF3B4A44"/>
             </rPr>
-            <t xml:space="preserve">Reuters 10月22日引述3名知情人士指出，台積電正調查半導體自動化設備使用低稀土或無稀土馬達的可能性，以降低部分設備供應受出口管制影響。報導指出供應商洽詢尚處早期，未有廣泛導入；台積電拒絕評論。稀土永磁材料可用於精密定位與自動化設備馬達，連結晶圓廠產線零組件與設備維護。報導所述風險來源為中國既有稀土及磁材出口管制，尚無特定台積電產線因短缺停工的證據。Reuters另引述工研院聲明，台灣正與經濟部產業技術司規劃稀土相關技術專案。工研院過去提及試量產線及供應目標屬先前政策背景，不能視為10月22日新增產能。未取得台積電直接公告，無供應商、馬達規格、設備替換數量或導入時間表；屬報導引述的評估。</t>
+            <t xml:space="preserve">Reuters 10 月 22 日引述 3 名知情人士指出，台積電正調查半導體自動化設備使用低稀土或無稀土馬達的可能性，以降低部分設備供應受出口管制影響。報導指出供應商洽詢尚處早期，未有廣泛導入；台積電拒絕評論。稀土永磁材料可用於精密定位與自動化設備馬達，連結晶圓廠產線零組件與設備維護。報導所述風險來源為中國既有稀土及磁材出口管制，尚無特定台積電產線因短缺停工的證據。Reuters 另引述工研院聲明，台灣正與經濟部產業技術司規劃稀土相關技術專案。工研院過去提及試量產線及供應目標屬先前政策背景，不能視為 10 月 22 日新增產能。未取得台積電直接公告，無供應商、馬達規格、設備替換數量或導入時間表；屬報導引述的評估。</t>
           </r>
         </is>
       </c>
@@ -569,7 +569,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="214" customHeight="1">
+    <row r="7" ht="230" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">05</t>
@@ -584,16 +584,16 @@
               <rFont val="PingFang TC"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">NVIDIA推出DSX POD模組化AI機房，鴻海與台灣ODM列合作供應商
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="PingFang TC"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">NVIDIA 10月21日在德國柏林公布以Vera Rubin為核心的DSX POD模組化AI工廠參考設計，合作廠商包括鴻海鴻佰、台達電、技嘉、和碩、雲達及緯創。NVIDIA稱已備妥現場基礎設施的案場部署可由6個月縮短至最快14天，全球合作交付目標為2027年初。DSX POD將伺服器整機、配線、機櫃電源、網路與液冷管路的整合測試提前在工廠完成；交付後仍須案場電力、散熱與網路就緒。台灣合作廠商分布在ODM、電源與機櫃系統。所稱14天為NVIDIA參考設計在已備妥案場條件下的最快目標，6個月為其比較情境，非所有專案實績。公司未列個別台廠供貨量與認證時程。個別客戶訂單、機櫃實際額定電力、液冷驗收、部署現場、交付數量均未公布。地點：德國柏林 GTC 開發者大會（發布會場）；模組化機房實際專案場址尚未公布。</t>
+            <t xml:space="preserve">NVIDIA 推出 DSX POD 模組化 AI 機房，鴻海與台灣 ODM 列合作供應商
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="PingFang TC"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">NVIDIA 10 月 21 日在德國柏林公布以 Vera Rubin 為核心的 DSX POD 模組化 AI 工廠參考設計，合作廠商包括鴻海鴻佰、台達電、技嘉、和碩、雲達及緯創。NVIDIA 稱已備妥現場基礎設施的案場部署可由 6 個月縮短至最快 14 天，全球合作交付目標為 2027 年初。DSX POD 將伺服器整機、配線、機櫃電源、網路與液冷管路的整合測試提前在工廠完成；交付後仍須案場電力、散熱與網路就緒。台灣合作廠商分布在 ODM、電源與機櫃系統。所稱 14 天為 NVIDIA 參考設計在已備妥案場條件下的最快目標，6 個月為其比較情境，非所有專案實績。公司未列個別台廠供貨量與認證時程。個別客戶訂單、機櫃實際額定電力、液冷驗收、部署現場、交付數量均未公布。地點：德國柏林 GTC 開發者大會（發布會場）；模組化機房實際專案場址尚未公布。</t>
           </r>
         </is>
       </c>
@@ -602,11 +602,11 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">資料中心電源轉換、液冷CDU、機櫃測試業者可核實箱體出廠的功能驗證範圍、現場變電與散熱介面，以及各ODM責任分工。最短部署時間仍是估計，尚無可比較的實際交付數據。</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="198" customHeight="1">
+          <t xml:space="preserve">資料中心電源轉換、液冷 CDU、機櫃測試業者可核實箱體出廠的功能驗證範圍、現場變電與散熱介面，以及各 ODM 責任分工。最短部署時間仍是估計，尚無可比較的實際交付數據。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="214" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">06</t>
@@ -621,16 +621,16 @@
               <rFont val="PingFang TC"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">馬來西亞SkyeChip與日本SAIMEMORY合作ZAM新型AI記憶體設計
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="PingFang TC"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">日本SAIMEMORY與馬來西亞SkyeChip於10月21日宣布設計工程合作，由SkyeChip提供記憶體介面、矽晶片設計及客製化IP，參與面向AI資料中心的Z-Angle Memory（ZAM）開發。官方公告未提供原型測試結果、記憶體頻寬或量產時程。SAIMEMORY為SoftBank旗下技術公司，ZAM定位為高容量、高頻寬及降低功耗的記憶體架構；SkyeChip提供IP設計、驗證與整合能力。這是新型記憶體研發合作，尚未等同HBM產線建成。合作在日本NEDO補助的Post-5G基礎設施研發計畫下進行。官方公告著重工程支援與未來商業化意向，未披露交付規格和產線資本支出。ZAM原型良率、傳輸頻寬、功耗測試、客戶樣品及商業量產日期尚未公布。</t>
+            <t xml:space="preserve">馬來西亞 SkyeChip 與日本 SAIMEMORY 合作 ZAM 新型 AI 記憶體設計
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="PingFang TC"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">日本 SAIMEMORY 與馬來西亞 SkyeChip 於 10 月 21 日宣布設計工程合作，由 SkyeChip 提供記憶體介面、矽晶片設計及客製化 IP，參與面向 AI 資料中心的 Z-Angle Memory（ZAM）開發。官方公告未提供原型測試結果、記憶體頻寬或量產時程。SAIMEMORY 為 SoftBank 旗下技術公司，ZAM 定位為高容量、高頻寬及降低功耗的記憶體架構；SkyeChip 提供 IP 設計、驗證與整合能力。這是新型記憶體研發合作，尚未等同 HBM 產線建成。合作在日本 NEDO 補助的 Post-5G 基礎設施研發計畫下進行。官方公告著重工程支援與未來商業化意向，未披露交付規格和產線資本支出。ZAM 原型良率、傳輸頻寬、功耗測試、客戶樣品及商業量產日期尚未公布。</t>
           </r>
         </is>
       </c>
@@ -639,11 +639,11 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">記憶體電源、測試及高速介面供應商應查詢ZAM的實際電壓、頻寬、封裝介面與驗證方法。現階段缺少樣品量產、封裝基板及測試產能資訊。</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="162" customHeight="1">
+          <t xml:space="preserve">記憶體電源、測試及高速介面供應商應查詢 ZAM 的實際電壓、頻寬、封裝介面與驗證方法。現階段缺少樣品量產、封裝基板及測試產能資訊。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="178" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">07</t>
@@ -658,16 +658,16 @@
               <rFont val="PingFang TC"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">台綜院：9月半導體用電首破45億度，年增11.55%
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="PingFang TC"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">台灣綜合研究院10月21日公布，2026年9月台灣半導體業用電量首次突破45億度，較去年同期增加11.55%；製造業高壓以上用電年增1.96%。台綜院預估全年半導體用電超過500億度，屬研究機構估計，並非全年已發生實績。半導體用電涵蓋晶圓、封裝與公用廠務負載，可作為生產活動的間接參考，但用電升高亦可能來自新廠試產、設備配置與能效因素，不能直接換算晶圓出貨。台綜院同時公布9月全國高壓以上產業用電年增1.76%，半導體分項年增11.55%；其2026全年500億度估計尚待後續實際統計驗證。未取得研究院原始月報表，各產業用電分項基期度數、個別廠區負載及全年實際用量無法核對。</t>
+            <t xml:space="preserve">台綜院：9 月半導體用電首破 45 億度，年增 11.55%
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="PingFang TC"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">台灣綜合研究院 10 月 21 日公布，2026 年 9 月台灣半導體業用電量首次突破 45 億度，較去年同期增加 11.55%；製造業高壓以上用電年增 1.96%。台綜院預估全年半導體用電超過 500 億度，屬研究機構估計，並非全年已發生實績。半導體用電涵蓋晶圓、封裝與公用廠務負載，可作為生產活動的間接參考，但用電升高亦可能來自新廠試產、設備配置與能效因素，不能直接換算晶圓出貨。台綜院同時公布 9 月全國高壓以上產業用電年增 1.76%，半導體分項年增 11.55%；其 2026 全年 500 億度估計尚待後續實際統計驗證。未取得研究院原始月報表，各產業用電分項基期度數、個別廠區負載及全年實際用量無法核對。</t>
           </r>
         </is>
       </c>
@@ -680,7 +680,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="178" customHeight="1">
+    <row r="10" ht="194" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">08</t>
@@ -695,16 +695,16 @@
               <rFont val="PingFang TC"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">馬國國會披露半導體培訓核准4,767萬令吉，涵蓋1.9萬名額
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="PingFang TC"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">馬來西亞貿工部長10月22日經媒體報導向國會指出，HRD Corp已於8月核准4,767萬令吉高科技培訓補助，涵蓋19,084個名額及9類半導體相關技能。截至2026年第3季，累計已有22,849名勞工完成各項相關訓練；這些數字各屬不同統計期間，不能直接相減作為未完成名額。培訓項目涵蓋IC設計、先進封裝、自動化及數位技術，是國家半導體策略人力供給的一環。2030年6萬名高技能工程師是政策目標，不能視為已受訓人數。依The Star引述，款項是在2026年8月獲核准；10月22日的新資訊為國會披露最新累計訓練進度。官方國會紀錄及核准項目細表未取得。未取得國會逐字稿、各訓練方案完訓率、實際支出及人才投入半導體公司的比例。</t>
+            <t xml:space="preserve">馬國國會披露半導體培訓核准 4,767 萬令吉，涵蓋 1.9 萬名額
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="PingFang TC"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">馬來西亞貿工部長 10 月 22 日經媒體報導向國會指出，HRD Corp 已於 8 月核准 4,767 萬令吉高科技培訓補助，涵蓋 19,084 個名額及 9 類半導體相關技能。截至 2026 年第 3 季，累計已有 22,849 名勞工完成各項相關訓練；這些數字各屬不同統計期間，不能直接相減作為未完成名額。培訓項目涵蓋 IC 設計、先進封裝、自動化及數位技術，是國家半導體策略人力供給的一環。2030 年 6 萬名高技能工程師是政策目標，不能視為已受訓人數。依 The Star 引述，款項是在 2026 年 8 月獲核准；10 月 22 日的新資訊為國會披露最新累計訓練進度。官方國會紀錄及核准項目細表未取得。未取得國會逐字稿、各訓練方案完訓率、實際支出及人才投入半導體公司的比例。</t>
           </r>
         </is>
       </c>

</xml_diff>